<commit_message>
fix: AudioFuse Studio の価格・Digiface AES の光入力・Volt 1/176 の同梱ソフトを修正
PR #57 のレビュー指摘への対応。

- AudioFuse Studio: 行の仕様 (ゲイン 71 dB / DR 118 dBA) は第 1 世代のため、
  参考価格を第 1 世代の公式出荷告知の 999 に戻す (1199 は Rev2 の価格)
- Digiface AES: 取扱説明書の Digital Inputs (ADAT Optical 1 x TOSLINK) に
  合わせて Optical Ports (Input) を 1 にし、Notes の 16ch・非対称の記述を修正
- Volt 1 / 176: Bundled Software を公式の同梱一覧 (Volt 2 / 4 / 476 と同一) に更新

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/audio_interfaces.xlsx
+++ b/data/audio_interfaces.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5268" uniqueCount="1918">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5268" uniqueCount="1917">
   <si>
     <t>Brand</t>
   </si>
@@ -4145,7 +4145,7 @@
     <t>TotalMix FX, DigiCheck NG, TotalMix Remote</t>
   </si>
   <si>
-    <t>14 input / 16 output total channels (analog+digital). 2 XLR combo mic/line inputs (75dB gain, individually switchable 48V phantom + PAD). 2 balanced XLR line outputs + 1 TRS phones output. ADAT is asymmetric: 2x TOSLINK input ports (16ch@48kHz) but only 1x TOSLINK output port (8ch@48kHz). SteadyClock FS, built-in sample rate converter, full standalone operation, bus-powered or external 12V supply.</t>
+    <t>14 input / 16 output total channels (analog+digital). 2 XLR combo mic/line inputs (75dB gain, individually switchable 48V phantom + PAD). 2 balanced XLR line outputs + 1 TRS phones output. 1x TOSLINK optical input and 1x TOSLINK optical output (ADAT 8ch@48kHz, or optical S/PDIF). SteadyClock FS, built-in sample rate converter, full standalone operation, bus-powered or external 12V supply.</t>
   </si>
   <si>
     <t>https://rme-audio.de/digiface-aes.html</t>
@@ -5150,7 +5150,7 @@
     <t>-102.5dB (0.00075%)</t>
   </si>
   <si>
-    <t>LUNA</t>
+    <t>LUNA, UA plugin bundle (13 titles), Melodyne Essential, Ampeg SVT-VR Classic Bass Bundle, UJAM Virtual Drummer DEEP, UJAM Virtual Bassist DANDY, Splice INSTRUMENT</t>
   </si>
   <si>
     <t>610 preamp</t>
@@ -5175,9 +5175,6 @@
   </si>
   <si>
     <t>-103.1dB (0.00070%)</t>
-  </si>
-  <si>
-    <t>LUNA, UA plugin bundle (13 titles), Melodyne Essential, Ampeg SVT-VR Classic Bass Bundle, UJAM Virtual Drummer DEEP, UJAM Virtual Bassist DANDY, Splice INSTRUMENT</t>
   </si>
   <si>
     <t>610 preamp mode (1176 as bundled plugin)</t>
@@ -10610,7 +10607,7 @@
         <v>257</v>
       </c>
       <c r="D58">
-        <v>1199</v>
+        <v>999</v>
       </c>
       <c r="E58">
         <v>4</v>
@@ -25793,7 +25790,7 @@
         <v>8</v>
       </c>
       <c r="J256">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K256">
         <v>1</v>
@@ -31123,13 +31120,13 @@
         <v>282</v>
       </c>
       <c r="AN326" t="s">
+        <v>1710</v>
+      </c>
+      <c r="AO326" t="s">
         <v>1719</v>
       </c>
-      <c r="AO326" t="s">
+      <c r="AP326" t="s">
         <v>1720</v>
-      </c>
-      <c r="AP326" t="s">
-        <v>1721</v>
       </c>
       <c r="AS326" t="s">
         <v>1713</v>
@@ -31140,7 +31137,7 @@
         <v>1653</v>
       </c>
       <c r="B327" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="C327" t="s">
         <v>271</v>
@@ -31203,16 +31200,16 @@
         <v>282</v>
       </c>
       <c r="AN327" t="s">
+        <v>1722</v>
+      </c>
+      <c r="AO327" t="s">
         <v>1723</v>
       </c>
-      <c r="AO327" t="s">
+      <c r="AP327" t="s">
         <v>1724</v>
       </c>
-      <c r="AP327" t="s">
+      <c r="AS327" t="s">
         <v>1725</v>
-      </c>
-      <c r="AS327" t="s">
-        <v>1726</v>
       </c>
     </row>
     <row r="328" spans="1:45" x14ac:dyDescent="0.25">
@@ -31220,7 +31217,7 @@
         <v>1653</v>
       </c>
       <c r="B328" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="C328" t="s">
         <v>271</v>
@@ -31289,16 +31286,16 @@
         <v>282</v>
       </c>
       <c r="AN328" t="s">
-        <v>1719</v>
+        <v>1710</v>
       </c>
       <c r="AO328" t="s">
+        <v>1727</v>
+      </c>
+      <c r="AP328" t="s">
         <v>1728</v>
       </c>
-      <c r="AP328" t="s">
+      <c r="AS328" t="s">
         <v>1729</v>
-      </c>
-      <c r="AS328" t="s">
-        <v>1730</v>
       </c>
     </row>
     <row r="329" spans="1:45" x14ac:dyDescent="0.25">
@@ -31306,7 +31303,7 @@
         <v>1653</v>
       </c>
       <c r="B329" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="C329" t="s">
         <v>271</v>
@@ -31381,16 +31378,16 @@
         <v>54</v>
       </c>
       <c r="AN329" t="s">
-        <v>1719</v>
+        <v>1710</v>
       </c>
       <c r="AO329" t="s">
         <v>387</v>
       </c>
       <c r="AP329" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="AS329" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="330" spans="1:45" x14ac:dyDescent="0.25">
@@ -31398,7 +31395,7 @@
         <v>1653</v>
       </c>
       <c r="B330" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="C330" t="s">
         <v>271</v>
@@ -31464,13 +31461,13 @@
         <v>282</v>
       </c>
       <c r="AO330" t="s">
+        <v>1733</v>
+      </c>
+      <c r="AP330" t="s">
         <v>1734</v>
       </c>
-      <c r="AP330" t="s">
-        <v>1735</v>
-      </c>
       <c r="AS330" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="331" spans="1:45" x14ac:dyDescent="0.25">
@@ -31478,7 +31475,7 @@
         <v>1653</v>
       </c>
       <c r="B331" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="C331" t="s">
         <v>257</v>
@@ -31523,7 +31520,7 @@
         <v>237</v>
       </c>
       <c r="V331" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
       <c r="W331">
         <v>192</v>
@@ -31559,30 +31556,30 @@
         <v>487</v>
       </c>
       <c r="AI331" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="AM331" t="s">
         <v>291</v>
       </c>
       <c r="AN331" t="s">
+        <v>1738</v>
+      </c>
+      <c r="AO331" t="s">
         <v>1739</v>
       </c>
-      <c r="AO331" t="s">
+      <c r="AP331" t="s">
         <v>1740</v>
       </c>
-      <c r="AP331" t="s">
+      <c r="AS331" t="s">
         <v>1741</v>
-      </c>
-      <c r="AS331" t="s">
-        <v>1742</v>
       </c>
     </row>
     <row r="332" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
+        <v>1742</v>
+      </c>
+      <c r="B332" t="s">
         <v>1743</v>
-      </c>
-      <c r="B332" t="s">
-        <v>1744</v>
       </c>
       <c r="C332" t="s">
         <v>381</v>
@@ -31633,24 +31630,24 @@
         <v>282</v>
       </c>
       <c r="AN332" t="s">
+        <v>1744</v>
+      </c>
+      <c r="AO332" t="s">
         <v>1745</v>
       </c>
-      <c r="AO332" t="s">
+      <c r="AP332" t="s">
         <v>1746</v>
       </c>
-      <c r="AP332" t="s">
+      <c r="AS332" t="s">
         <v>1747</v>
-      </c>
-      <c r="AS332" t="s">
-        <v>1748</v>
       </c>
     </row>
     <row r="333" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B333" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="C333" t="s">
         <v>381</v>
@@ -31701,27 +31698,27 @@
         <v>282</v>
       </c>
       <c r="AN333" t="s">
-        <v>1745</v>
+        <v>1744</v>
       </c>
       <c r="AO333" t="s">
+        <v>1749</v>
+      </c>
+      <c r="AP333" t="s">
         <v>1750</v>
       </c>
-      <c r="AP333" t="s">
-        <v>1751</v>
-      </c>
       <c r="AQ333">
         <v>2</v>
       </c>
       <c r="AS333" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
     </row>
     <row r="334" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B334" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="C334" t="s">
         <v>381</v>
@@ -31772,27 +31769,27 @@
         <v>282</v>
       </c>
       <c r="AN334" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AO334" t="s">
         <v>1753</v>
       </c>
-      <c r="AO334" t="s">
+      <c r="AP334" t="s">
         <v>1754</v>
       </c>
-      <c r="AP334" t="s">
+      <c r="AQ334">
+        <v>2</v>
+      </c>
+      <c r="AS334" t="s">
         <v>1755</v>
-      </c>
-      <c r="AQ334">
-        <v>2</v>
-      </c>
-      <c r="AS334" t="s">
-        <v>1756</v>
       </c>
     </row>
     <row r="335" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B335" t="s">
-        <v>1757</v>
+        <v>1756</v>
       </c>
       <c r="C335" t="s">
         <v>47</v>
@@ -31852,24 +31849,24 @@
         <v>54</v>
       </c>
       <c r="AN335" t="s">
+        <v>1757</v>
+      </c>
+      <c r="AO335" t="s">
         <v>1758</v>
       </c>
-      <c r="AO335" t="s">
+      <c r="AP335" t="s">
         <v>1759</v>
       </c>
-      <c r="AP335" t="s">
+      <c r="AS335" t="s">
         <v>1760</v>
-      </c>
-      <c r="AS335" t="s">
-        <v>1761</v>
       </c>
     </row>
     <row r="336" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B336" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="C336" t="s">
         <v>47</v>
@@ -31929,24 +31926,24 @@
         <v>54</v>
       </c>
       <c r="AN336" t="s">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="AO336" t="s">
-        <v>1763</v>
+        <v>1762</v>
       </c>
       <c r="AP336" t="s">
+        <v>1759</v>
+      </c>
+      <c r="AS336" t="s">
         <v>1760</v>
-      </c>
-      <c r="AS336" t="s">
-        <v>1761</v>
       </c>
     </row>
     <row r="337" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B337" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="C337" t="s">
         <v>47</v>
@@ -31991,27 +31988,27 @@
         <v>54</v>
       </c>
       <c r="AN337" t="s">
-        <v>1753</v>
+        <v>1752</v>
       </c>
       <c r="AO337" t="s">
+        <v>1764</v>
+      </c>
+      <c r="AP337" t="s">
         <v>1765</v>
-      </c>
-      <c r="AP337" t="s">
-        <v>1766</v>
       </c>
       <c r="AQ337">
         <v>4</v>
       </c>
       <c r="AS337" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
     </row>
     <row r="338" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B338" t="s">
-        <v>1768</v>
+        <v>1767</v>
       </c>
       <c r="C338" t="s">
         <v>47</v>
@@ -32053,27 +32050,27 @@
         <v>54</v>
       </c>
       <c r="AN338" t="s">
-        <v>1753</v>
+        <v>1752</v>
       </c>
       <c r="AO338" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="AP338" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="AQ338">
         <v>4</v>
       </c>
       <c r="AS338" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
     </row>
     <row r="339" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B339" t="s">
-        <v>1770</v>
+        <v>1769</v>
       </c>
       <c r="C339" t="s">
         <v>47</v>
@@ -32127,24 +32124,24 @@
         <v>54</v>
       </c>
       <c r="AO339" t="s">
-        <v>1771</v>
+        <v>1770</v>
       </c>
       <c r="AP339" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="AQ339">
         <v>4</v>
       </c>
       <c r="AS339" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="340" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B340" t="s">
-        <v>1773</v>
+        <v>1772</v>
       </c>
       <c r="C340" t="s">
         <v>47</v>
@@ -32195,24 +32192,24 @@
         <v>54</v>
       </c>
       <c r="AO340" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="AP340" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="AQ340">
         <v>4</v>
       </c>
       <c r="AS340" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="341" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B341" t="s">
-        <v>1775</v>
+        <v>1774</v>
       </c>
       <c r="C341" t="s">
         <v>47</v>
@@ -32263,27 +32260,27 @@
         <v>54</v>
       </c>
       <c r="AN341" t="s">
-        <v>1753</v>
+        <v>1752</v>
       </c>
       <c r="AO341" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
       <c r="AP341" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="AQ341">
         <v>4</v>
       </c>
       <c r="AS341" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="342" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B342" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="C342" t="s">
         <v>47</v>
@@ -32337,24 +32334,24 @@
         <v>54</v>
       </c>
       <c r="AO342" t="s">
-        <v>1779</v>
+        <v>1778</v>
       </c>
       <c r="AP342" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="AQ342">
         <v>4</v>
       </c>
       <c r="AS342" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="343" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B343" t="s">
-        <v>1780</v>
+        <v>1779</v>
       </c>
       <c r="C343" t="s">
         <v>47</v>
@@ -32402,7 +32399,7 @@
         <v>48</v>
       </c>
       <c r="AD343" t="s">
-        <v>1781</v>
+        <v>1780</v>
       </c>
       <c r="AG343" t="s">
         <v>1190</v>
@@ -32417,27 +32414,27 @@
         <v>54</v>
       </c>
       <c r="AN343" t="s">
+        <v>1781</v>
+      </c>
+      <c r="AO343" t="s">
         <v>1782</v>
       </c>
-      <c r="AO343" t="s">
+      <c r="AP343" t="s">
         <v>1783</v>
-      </c>
-      <c r="AP343" t="s">
-        <v>1784</v>
       </c>
       <c r="AQ343">
         <v>4</v>
       </c>
       <c r="AS343" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="344" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B344" t="s">
-        <v>1786</v>
+        <v>1785</v>
       </c>
       <c r="C344" t="s">
         <v>47</v>
@@ -32485,7 +32482,7 @@
         <v>48</v>
       </c>
       <c r="AD344" t="s">
-        <v>1781</v>
+        <v>1780</v>
       </c>
       <c r="AF344" t="s">
         <v>1190</v>
@@ -32500,24 +32497,24 @@
         <v>54</v>
       </c>
       <c r="AO344" t="s">
+        <v>1786</v>
+      </c>
+      <c r="AP344" t="s">
         <v>1787</v>
-      </c>
-      <c r="AP344" t="s">
-        <v>1788</v>
       </c>
       <c r="AQ344">
         <v>4</v>
       </c>
       <c r="AS344" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="345" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B345" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="C345" t="s">
         <v>47</v>
@@ -32565,7 +32562,7 @@
         <v>48</v>
       </c>
       <c r="AD345" t="s">
-        <v>1781</v>
+        <v>1780</v>
       </c>
       <c r="AG345" t="s">
         <v>1190</v>
@@ -32580,24 +32577,24 @@
         <v>54</v>
       </c>
       <c r="AO345" t="s">
+        <v>1789</v>
+      </c>
+      <c r="AP345" t="s">
         <v>1790</v>
-      </c>
-      <c r="AP345" t="s">
-        <v>1791</v>
       </c>
       <c r="AQ345">
         <v>4</v>
       </c>
       <c r="AS345" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="346" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B346" t="s">
-        <v>1792</v>
+        <v>1791</v>
       </c>
       <c r="C346" t="s">
         <v>47</v>
@@ -32645,7 +32642,7 @@
         <v>48</v>
       </c>
       <c r="AD346" t="s">
-        <v>1781</v>
+        <v>1780</v>
       </c>
       <c r="AF346" t="s">
         <v>1190</v>
@@ -32660,27 +32657,27 @@
         <v>54</v>
       </c>
       <c r="AN346" t="s">
+        <v>1792</v>
+      </c>
+      <c r="AO346" t="s">
         <v>1793</v>
       </c>
-      <c r="AO346" t="s">
+      <c r="AP346" t="s">
         <v>1794</v>
-      </c>
-      <c r="AP346" t="s">
-        <v>1795</v>
       </c>
       <c r="AQ346">
         <v>4</v>
       </c>
       <c r="AS346" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="347" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B347" t="s">
-        <v>1796</v>
+        <v>1795</v>
       </c>
       <c r="C347" t="s">
         <v>205</v>
@@ -32710,7 +32707,7 @@
         <v>24</v>
       </c>
       <c r="Y347" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="AF347" t="s">
         <v>362</v>
@@ -32722,24 +32719,24 @@
         <v>54</v>
       </c>
       <c r="AN347" t="s">
+        <v>1797</v>
+      </c>
+      <c r="AO347" t="s">
         <v>1798</v>
       </c>
-      <c r="AO347" t="s">
+      <c r="AP347" t="s">
         <v>1799</v>
       </c>
-      <c r="AP347" t="s">
+      <c r="AS347" t="s">
         <v>1800</v>
-      </c>
-      <c r="AS347" t="s">
-        <v>1801</v>
       </c>
     </row>
     <row r="348" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B348" t="s">
-        <v>1802</v>
+        <v>1801</v>
       </c>
       <c r="C348" t="s">
         <v>297</v>
@@ -32802,24 +32799,24 @@
         <v>54</v>
       </c>
       <c r="AN348" t="s">
+        <v>1802</v>
+      </c>
+      <c r="AO348" t="s">
         <v>1803</v>
       </c>
-      <c r="AO348" t="s">
+      <c r="AP348" t="s">
         <v>1804</v>
       </c>
-      <c r="AP348" t="s">
+      <c r="AS348" t="s">
         <v>1805</v>
-      </c>
-      <c r="AS348" t="s">
-        <v>1806</v>
       </c>
     </row>
     <row r="349" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B349" t="s">
-        <v>1807</v>
+        <v>1806</v>
       </c>
       <c r="C349" t="s">
         <v>297</v>
@@ -32879,24 +32876,24 @@
         <v>54</v>
       </c>
       <c r="AN349" t="s">
+        <v>1802</v>
+      </c>
+      <c r="AO349" t="s">
         <v>1803</v>
       </c>
-      <c r="AO349" t="s">
-        <v>1804</v>
-      </c>
       <c r="AP349" t="s">
+        <v>1807</v>
+      </c>
+      <c r="AS349" t="s">
         <v>1808</v>
-      </c>
-      <c r="AS349" t="s">
-        <v>1809</v>
       </c>
     </row>
     <row r="350" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B350" t="s">
-        <v>1810</v>
+        <v>1809</v>
       </c>
       <c r="C350" t="s">
         <v>271</v>
@@ -32932,7 +32929,7 @@
         <v>32</v>
       </c>
       <c r="Y350" t="s">
-        <v>1811</v>
+        <v>1810</v>
       </c>
       <c r="AB350" t="s">
         <v>73</v>
@@ -32950,7 +32947,7 @@
         <v>1365</v>
       </c>
       <c r="AI350" t="s">
-        <v>1812</v>
+        <v>1811</v>
       </c>
       <c r="AK350" t="s">
         <v>266</v>
@@ -32959,24 +32956,24 @@
         <v>54</v>
       </c>
       <c r="AN350" t="s">
+        <v>1812</v>
+      </c>
+      <c r="AO350" t="s">
         <v>1813</v>
       </c>
-      <c r="AO350" t="s">
+      <c r="AP350" t="s">
         <v>1814</v>
       </c>
-      <c r="AP350" t="s">
+      <c r="AS350" t="s">
         <v>1815</v>
-      </c>
-      <c r="AS350" t="s">
-        <v>1816</v>
       </c>
     </row>
     <row r="351" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B351" t="s">
-        <v>1817</v>
+        <v>1816</v>
       </c>
       <c r="C351" t="s">
         <v>271</v>
@@ -33009,7 +33006,7 @@
         <v>32</v>
       </c>
       <c r="Y351" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
       <c r="Z351" t="s">
         <v>272</v>
@@ -33039,24 +33036,24 @@
         <v>54</v>
       </c>
       <c r="AN351" t="s">
+        <v>1818</v>
+      </c>
+      <c r="AO351" t="s">
         <v>1819</v>
       </c>
-      <c r="AO351" t="s">
+      <c r="AP351" t="s">
         <v>1820</v>
       </c>
-      <c r="AP351" t="s">
+      <c r="AS351" t="s">
         <v>1821</v>
-      </c>
-      <c r="AS351" t="s">
-        <v>1822</v>
       </c>
     </row>
     <row r="352" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B352" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="C352" t="s">
         <v>271</v>
@@ -33092,7 +33089,7 @@
         <v>32</v>
       </c>
       <c r="Y352" t="s">
-        <v>1811</v>
+        <v>1810</v>
       </c>
       <c r="AB352" t="s">
         <v>73</v>
@@ -33110,7 +33107,7 @@
         <v>1365</v>
       </c>
       <c r="AI352" t="s">
-        <v>1812</v>
+        <v>1811</v>
       </c>
       <c r="AK352" t="s">
         <v>266</v>
@@ -33119,24 +33116,24 @@
         <v>54</v>
       </c>
       <c r="AN352" t="s">
-        <v>1813</v>
+        <v>1812</v>
       </c>
       <c r="AO352" t="s">
+        <v>1823</v>
+      </c>
+      <c r="AP352" t="s">
         <v>1824</v>
       </c>
-      <c r="AP352" t="s">
+      <c r="AS352" t="s">
         <v>1825</v>
-      </c>
-      <c r="AS352" t="s">
-        <v>1826</v>
       </c>
     </row>
     <row r="353" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B353" t="s">
-        <v>1827</v>
+        <v>1826</v>
       </c>
       <c r="C353" t="s">
         <v>271</v>
@@ -33172,7 +33169,7 @@
         <v>32</v>
       </c>
       <c r="Y353" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
       <c r="Z353" t="s">
         <v>272</v>
@@ -33184,7 +33181,7 @@
         <v>73</v>
       </c>
       <c r="AC353" t="s">
-        <v>1828</v>
+        <v>1827</v>
       </c>
       <c r="AD353">
         <v>54</v>
@@ -33205,24 +33202,24 @@
         <v>54</v>
       </c>
       <c r="AN353" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="AO353" t="s">
+        <v>1828</v>
+      </c>
+      <c r="AP353" t="s">
         <v>1829</v>
       </c>
-      <c r="AP353" t="s">
+      <c r="AS353" t="s">
         <v>1830</v>
-      </c>
-      <c r="AS353" t="s">
-        <v>1831</v>
       </c>
     </row>
     <row r="354" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B354" t="s">
-        <v>1832</v>
+        <v>1831</v>
       </c>
       <c r="C354" t="s">
         <v>257</v>
@@ -33258,7 +33255,7 @@
         <v>32</v>
       </c>
       <c r="Y354" t="s">
-        <v>1811</v>
+        <v>1810</v>
       </c>
       <c r="AB354" t="s">
         <v>73</v>
@@ -33276,7 +33273,7 @@
         <v>1365</v>
       </c>
       <c r="AI354" t="s">
-        <v>1812</v>
+        <v>1811</v>
       </c>
       <c r="AK354" t="s">
         <v>266</v>
@@ -33285,24 +33282,24 @@
         <v>54</v>
       </c>
       <c r="AN354" t="s">
-        <v>1813</v>
+        <v>1812</v>
       </c>
       <c r="AO354" t="s">
+        <v>1832</v>
+      </c>
+      <c r="AP354" t="s">
         <v>1833</v>
       </c>
-      <c r="AP354" t="s">
+      <c r="AS354" t="s">
         <v>1834</v>
-      </c>
-      <c r="AS354" t="s">
-        <v>1835</v>
       </c>
     </row>
     <row r="355" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B355" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
       <c r="C355" t="s">
         <v>381</v>
@@ -33353,21 +33350,21 @@
         <v>54</v>
       </c>
       <c r="AN355" t="s">
+        <v>1836</v>
+      </c>
+      <c r="AO355" t="s">
         <v>1837</v>
       </c>
-      <c r="AO355" t="s">
+      <c r="AP355" t="s">
         <v>1838</v>
-      </c>
-      <c r="AP355" t="s">
-        <v>1839</v>
       </c>
     </row>
     <row r="356" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="B356" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="C356" t="s">
         <v>381</v>
@@ -33412,18 +33409,18 @@
         <v>54</v>
       </c>
       <c r="AO356" t="s">
+        <v>1840</v>
+      </c>
+      <c r="AP356" t="s">
         <v>1841</v>
-      </c>
-      <c r="AP356" t="s">
-        <v>1842</v>
       </c>
     </row>
     <row r="357" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B357" t="s">
         <v>1843</v>
-      </c>
-      <c r="B357" t="s">
-        <v>1844</v>
       </c>
       <c r="C357" t="s">
         <v>297</v>
@@ -33468,10 +33465,10 @@
         <v>48</v>
       </c>
       <c r="AD357" t="s">
+        <v>1844</v>
+      </c>
+      <c r="AK357" t="s">
         <v>1845</v>
-      </c>
-      <c r="AK357" t="s">
-        <v>1846</v>
       </c>
       <c r="AM357" t="s">
         <v>260</v>
@@ -33480,18 +33477,18 @@
         <v>742</v>
       </c>
       <c r="AP357" t="s">
+        <v>1846</v>
+      </c>
+      <c r="AS357" t="s">
         <v>1847</v>
-      </c>
-      <c r="AS357" t="s">
-        <v>1848</v>
       </c>
     </row>
     <row r="358" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B358" t="s">
-        <v>1849</v>
+        <v>1848</v>
       </c>
       <c r="C358" t="s">
         <v>297</v>
@@ -33533,7 +33530,7 @@
         <v>48</v>
       </c>
       <c r="AD358" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
       <c r="AK358">
         <v>-120</v>
@@ -33542,21 +33539,21 @@
         <v>763</v>
       </c>
       <c r="AO358" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="AP358" t="s">
+        <v>1846</v>
+      </c>
+      <c r="AS358" t="s">
         <v>1847</v>
-      </c>
-      <c r="AS358" t="s">
-        <v>1848</v>
       </c>
     </row>
     <row r="359" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B359" t="s">
-        <v>1852</v>
+        <v>1851</v>
       </c>
       <c r="C359" t="s">
         <v>297</v>
@@ -33598,30 +33595,30 @@
         <v>48</v>
       </c>
       <c r="AD359" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
       <c r="AK359" t="s">
-        <v>1846</v>
+        <v>1845</v>
       </c>
       <c r="AM359" t="s">
         <v>260</v>
       </c>
       <c r="AO359" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
       <c r="AP359" t="s">
+        <v>1846</v>
+      </c>
+      <c r="AS359" t="s">
         <v>1847</v>
-      </c>
-      <c r="AS359" t="s">
-        <v>1848</v>
       </c>
     </row>
     <row r="360" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B360" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
       <c r="C360" t="s">
         <v>47</v>
@@ -33669,7 +33666,7 @@
         <v>73</v>
       </c>
       <c r="AD360" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="AK360" t="s">
         <v>266</v>
@@ -33678,24 +33675,24 @@
         <v>54</v>
       </c>
       <c r="AO360" t="s">
+        <v>1855</v>
+      </c>
+      <c r="AP360" t="s">
         <v>1856</v>
-      </c>
-      <c r="AP360" t="s">
-        <v>1857</v>
       </c>
       <c r="AQ360">
         <v>4</v>
       </c>
       <c r="AS360" t="s">
-        <v>1858</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="361" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B361" t="s">
-        <v>1859</v>
+        <v>1858</v>
       </c>
       <c r="C361" t="s">
         <v>47</v>
@@ -33752,24 +33749,24 @@
         <v>282</v>
       </c>
       <c r="AO361" t="s">
+        <v>1859</v>
+      </c>
+      <c r="AP361" t="s">
         <v>1860</v>
-      </c>
-      <c r="AP361" t="s">
-        <v>1861</v>
       </c>
       <c r="AQ361">
         <v>4</v>
       </c>
       <c r="AS361" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="362" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B362" t="s">
-        <v>1863</v>
+        <v>1862</v>
       </c>
       <c r="C362" t="s">
         <v>47</v>
@@ -33817,33 +33814,33 @@
         <v>48</v>
       </c>
       <c r="AD362" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="AK362">
         <v>-128</v>
       </c>
       <c r="AM362" t="s">
+        <v>1863</v>
+      </c>
+      <c r="AO362" t="s">
         <v>1864</v>
       </c>
-      <c r="AO362" t="s">
+      <c r="AP362" t="s">
         <v>1865</v>
-      </c>
-      <c r="AP362" t="s">
-        <v>1866</v>
       </c>
       <c r="AQ362">
         <v>4</v>
       </c>
       <c r="AS362" t="s">
-        <v>1867</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="363" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B363" t="s">
-        <v>1868</v>
+        <v>1867</v>
       </c>
       <c r="C363" t="s">
         <v>47</v>
@@ -33894,27 +33891,27 @@
         <v>48</v>
       </c>
       <c r="AK363" t="s">
-        <v>1846</v>
+        <v>1845</v>
       </c>
       <c r="AM363" t="s">
         <v>260</v>
       </c>
       <c r="AO363" t="s">
+        <v>1868</v>
+      </c>
+      <c r="AP363" t="s">
         <v>1869</v>
       </c>
-      <c r="AP363" t="s">
+      <c r="AS363" t="s">
         <v>1870</v>
-      </c>
-      <c r="AS363" t="s">
-        <v>1871</v>
       </c>
     </row>
     <row r="364" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B364" t="s">
-        <v>1872</v>
+        <v>1871</v>
       </c>
       <c r="C364" t="s">
         <v>47</v>
@@ -33959,30 +33956,30 @@
         <v>73</v>
       </c>
       <c r="AD364" t="s">
+        <v>1872</v>
+      </c>
+      <c r="AK364" t="s">
         <v>1873</v>
-      </c>
-      <c r="AK364" t="s">
-        <v>1874</v>
       </c>
       <c r="AM364" t="s">
         <v>291</v>
       </c>
       <c r="AO364" t="s">
+        <v>1874</v>
+      </c>
+      <c r="AP364" t="s">
         <v>1875</v>
       </c>
-      <c r="AP364" t="s">
+      <c r="AS364" t="s">
         <v>1876</v>
-      </c>
-      <c r="AS364" t="s">
-        <v>1877</v>
       </c>
     </row>
     <row r="365" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B365" t="s">
-        <v>1878</v>
+        <v>1877</v>
       </c>
       <c r="C365" t="s">
         <v>47</v>
@@ -34027,30 +34024,30 @@
         <v>48</v>
       </c>
       <c r="AD365" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="AK365">
         <v>-128</v>
       </c>
       <c r="AM365" t="s">
-        <v>1864</v>
+        <v>1863</v>
       </c>
       <c r="AO365" t="s">
+        <v>1878</v>
+      </c>
+      <c r="AP365" t="s">
         <v>1879</v>
       </c>
-      <c r="AP365" t="s">
+      <c r="AS365" t="s">
         <v>1880</v>
-      </c>
-      <c r="AS365" t="s">
-        <v>1881</v>
       </c>
     </row>
     <row r="366" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B366" t="s">
-        <v>1882</v>
+        <v>1881</v>
       </c>
       <c r="C366" t="s">
         <v>47</v>
@@ -34104,21 +34101,21 @@
         <v>763</v>
       </c>
       <c r="AO366" t="s">
+        <v>1882</v>
+      </c>
+      <c r="AP366" t="s">
         <v>1883</v>
       </c>
-      <c r="AP366" t="s">
+      <c r="AS366" t="s">
         <v>1884</v>
-      </c>
-      <c r="AS366" t="s">
-        <v>1885</v>
       </c>
     </row>
     <row r="367" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B367" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="C367" t="s">
         <v>381</v>
@@ -34142,21 +34139,21 @@
         <v>54</v>
       </c>
       <c r="AN367" t="s">
+        <v>1886</v>
+      </c>
+      <c r="AO367" t="s">
         <v>1887</v>
       </c>
-      <c r="AO367" t="s">
+      <c r="AP367" t="s">
         <v>1888</v>
-      </c>
-      <c r="AP367" t="s">
-        <v>1889</v>
       </c>
     </row>
     <row r="368" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B368" t="s">
-        <v>1890</v>
+        <v>1889</v>
       </c>
       <c r="C368" t="s">
         <v>381</v>
@@ -34192,18 +34189,18 @@
         <v>260</v>
       </c>
       <c r="AO368" t="s">
+        <v>1890</v>
+      </c>
+      <c r="AP368" t="s">
         <v>1891</v>
-      </c>
-      <c r="AP368" t="s">
-        <v>1892</v>
       </c>
     </row>
     <row r="369" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B369" t="s">
-        <v>1893</v>
+        <v>1892</v>
       </c>
       <c r="C369" t="s">
         <v>381</v>
@@ -34236,7 +34233,7 @@
         <v>48</v>
       </c>
       <c r="AD369" t="s">
-        <v>1894</v>
+        <v>1893</v>
       </c>
       <c r="AK369">
         <v>-125</v>
@@ -34245,21 +34242,21 @@
         <v>763</v>
       </c>
       <c r="AO369" t="s">
+        <v>1894</v>
+      </c>
+      <c r="AP369" t="s">
         <v>1895</v>
       </c>
-      <c r="AP369" t="s">
+      <c r="AS369" t="s">
         <v>1896</v>
-      </c>
-      <c r="AS369" t="s">
-        <v>1897</v>
       </c>
     </row>
     <row r="370" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B370" t="s">
-        <v>1898</v>
+        <v>1897</v>
       </c>
       <c r="C370" t="s">
         <v>381</v>
@@ -34298,27 +34295,27 @@
         <v>70</v>
       </c>
       <c r="AK370" t="s">
-        <v>1899</v>
+        <v>1898</v>
       </c>
       <c r="AM370" t="s">
         <v>54</v>
       </c>
       <c r="AO370" t="s">
+        <v>1899</v>
+      </c>
+      <c r="AP370" t="s">
         <v>1900</v>
       </c>
-      <c r="AP370" t="s">
+      <c r="AS370" t="s">
         <v>1901</v>
-      </c>
-      <c r="AS370" t="s">
-        <v>1902</v>
       </c>
     </row>
     <row r="371" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B371" t="s">
-        <v>1903</v>
+        <v>1902</v>
       </c>
       <c r="C371" t="s">
         <v>297</v>
@@ -34360,7 +34357,7 @@
         <v>48</v>
       </c>
       <c r="AD371" t="s">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="AK371">
         <v>-119.5</v>
@@ -34372,24 +34369,24 @@
         <v>1428</v>
       </c>
       <c r="AO371" t="s">
+        <v>1904</v>
+      </c>
+      <c r="AP371" t="s">
         <v>1905</v>
       </c>
-      <c r="AP371" t="s">
+      <c r="AR371">
+        <v>2</v>
+      </c>
+      <c r="AS371" t="s">
         <v>1906</v>
-      </c>
-      <c r="AR371">
-        <v>2</v>
-      </c>
-      <c r="AS371" t="s">
-        <v>1907</v>
       </c>
     </row>
     <row r="372" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B372" t="s">
-        <v>1908</v>
+        <v>1907</v>
       </c>
       <c r="C372" t="s">
         <v>297</v>
@@ -34443,7 +34440,7 @@
         <v>48</v>
       </c>
       <c r="AD372" t="s">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="AK372">
         <v>-119.5</v>
@@ -34455,24 +34452,24 @@
         <v>1428</v>
       </c>
       <c r="AO372" t="s">
+        <v>1908</v>
+      </c>
+      <c r="AP372" t="s">
         <v>1909</v>
       </c>
-      <c r="AP372" t="s">
+      <c r="AR372">
+        <v>2</v>
+      </c>
+      <c r="AS372" t="s">
         <v>1910</v>
-      </c>
-      <c r="AR372">
-        <v>2</v>
-      </c>
-      <c r="AS372" t="s">
-        <v>1911</v>
       </c>
     </row>
     <row r="373" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="B373" t="s">
-        <v>1912</v>
+        <v>1911</v>
       </c>
       <c r="C373" t="s">
         <v>297</v>
@@ -34523,13 +34520,13 @@
         <v>282</v>
       </c>
       <c r="AO373" t="s">
+        <v>1912</v>
+      </c>
+      <c r="AP373" t="s">
         <v>1913</v>
       </c>
-      <c r="AP373" t="s">
+      <c r="AS373" t="s">
         <v>1914</v>
-      </c>
-      <c r="AS373" t="s">
-        <v>1915</v>
       </c>
     </row>
   </sheetData>
@@ -34551,7 +34548,7 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>1916</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -34604,7 +34601,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="B8">
         <v>216</v>

</xml_diff>

<commit_message>
fix: AudioFuse Studio の行を現行の Rev2 に切り替える
公式の製品ページ (Product Page URL の参照先) は Rev2 のみを扱っており、
行は第 1 世代の仕様と価格のままだった。公式 Details の値で Rev2 に更新する。

- Model: AudioFuse Studio → AudioFuse Studio Rev2
- Reference Price 999 → 1199、Preamp Gain Range 71 → 78
- Bundled Software と Notes を Rev2 の記載に更新
- Measurement Reports: 第 1 世代を測った ProSound を外し、
  メーカー公称の Details ページに差し替え

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/audio_interfaces.xlsx
+++ b/data/audio_interfaces.xlsx
@@ -1097,28 +1097,28 @@
     <t>[ProSound](https://prosound.ixbt.com/interfaces/arturia-8pre.shtml)</t>
   </si>
   <si>
-    <t>AudioFuse Studio</t>
+    <t>AudioFuse Studio Rev2</t>
   </si>
   <si>
     <t>USB-C (fully USB 2.0 compatible)</t>
   </si>
   <si>
-    <t>71</t>
+    <t>78</t>
   </si>
   <si>
     <t>118</t>
   </si>
   <si>
-    <t>AudioFuse Creative Suite (incl. Analog Lab Intro)</t>
-  </si>
-  <si>
-    <t>Bluetooth</t>
+    <t>AudioFuse Creative Suite (11 titles incl. Analog Lab Intro, Comp DIODE-609)</t>
+  </si>
+  <si>
+    <t>Rev2: optimized DiscretePRO preamps (mic max input +18dBu, boost +17dB); Bluetooth streaming (AAC, aptX, aptX HD, aptX Low Latency); inputs 5-6 switchable to phono/RIAA preamp; integrated 3-port USB 2 hub</t>
   </si>
   <si>
     <t>https://www.arturia.com/products/audio/audiofuse-studio/overview</t>
   </si>
   <si>
-    <t>[ProSound](https://prosound.ixbt.com/interfaces/arturia-studio.shtml)</t>
+    <t>[Manufacturer](https://www.arturia.com/products/audio/audiofuse-studio/details)</t>
   </si>
   <si>
     <t>MiniFuse 1</t>
@@ -10607,7 +10607,7 @@
         <v>257</v>
       </c>
       <c r="D58">
-        <v>999</v>
+        <v>1199</v>
       </c>
       <c r="E58">
         <v>4</v>

</xml_diff>